<commit_message>
Separate tribal ownerships and add to Other group
</commit_message>
<xml_diff>
--- a/tables/ownership_summary.xlsx
+++ b/tables/ownership_summary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\ORISE\Projects\salvage\pfh\tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E58F44B-3A45-456A-9756-CA74BA38B981}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BF14C29-BE0F-43DA-90F0-9B3CDF0D9979}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="7980" xr2:uid="{7179679D-7B0A-430B-92F9-F823978B3D0B}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Owner</t>
   </si>
@@ -58,6 +58,12 @@
   </si>
   <si>
     <t>Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Tribal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    State/local</t>
   </si>
 </sst>
 </file>
@@ -67,7 +73,7 @@
   <numFmts count="3">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="168" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -130,15 +136,15 @@
   <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
@@ -456,9 +462,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA33F950-9190-41C7-9FDF-D97890B656D3}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.7109375" bestFit="1" customWidth="1"/>
@@ -487,18 +494,18 @@
         <v>5</v>
       </c>
       <c r="B2" s="2">
-        <v>79898</v>
+        <v>79815</v>
       </c>
       <c r="C2" s="2">
-        <v>1634944</v>
+        <v>1632784</v>
       </c>
       <c r="D2" s="1">
         <f>B2/C2</f>
-        <v>4.886895208643232E-2</v>
+        <v>4.8882767102078416E-2</v>
       </c>
       <c r="E2" s="4">
-        <f>C2/$C$7</f>
-        <v>0.7326570550121061</v>
+        <f>C2/$C$9</f>
+        <v>0.7320158294146103</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -506,18 +513,18 @@
         <v>6</v>
       </c>
       <c r="B3" s="6">
-        <v>71706</v>
+        <v>71690</v>
       </c>
       <c r="C3" s="6">
-        <v>1458084</v>
+        <v>1457159</v>
       </c>
       <c r="D3" s="7">
-        <f t="shared" ref="D3:D7" si="0">B3/C3</f>
-        <v>4.9178236644802358E-2</v>
+        <f t="shared" ref="D3:D9" si="0">B3/C3</f>
+        <v>4.9198474565919026E-2</v>
       </c>
       <c r="E3" s="8">
-        <f>C3/$C$7</f>
-        <v>0.65340190820008004</v>
+        <f>C3/$C$9</f>
+        <v>0.65327897258545164</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -525,18 +532,18 @@
         <v>7</v>
       </c>
       <c r="B4" s="6">
-        <v>8165</v>
+        <v>8097</v>
       </c>
       <c r="C4" s="6">
-        <v>175666</v>
+        <v>174431</v>
       </c>
       <c r="D4" s="7">
         <f t="shared" si="0"/>
-        <v>4.6480252296972661E-2</v>
+        <v>4.6419501120787014E-2</v>
       </c>
       <c r="E4" s="8">
-        <f>C4/$C$7</f>
-        <v>7.8720087186935225E-2</v>
+        <f>C4/$C$9</f>
+        <v>7.8201558283655326E-2</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -544,18 +551,18 @@
         <v>8</v>
       </c>
       <c r="B5" s="2">
-        <v>93798</v>
+        <v>88536</v>
       </c>
       <c r="C5" s="2">
-        <v>538530</v>
+        <v>475115</v>
       </c>
       <c r="D5" s="1">
-        <f t="shared" si="0"/>
-        <v>0.17417414071639464</v>
+        <f>B5/C5</f>
+        <v>0.18634646348778716</v>
       </c>
       <c r="E5" s="4">
-        <f>C5/$C$7</f>
-        <v>0.24132802336695905</v>
+        <f>C5/$C$9</f>
+        <v>0.21300533370753422</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -563,37 +570,77 @@
         <v>9</v>
       </c>
       <c r="B6" s="2">
-        <v>4008</v>
+        <v>9338</v>
       </c>
       <c r="C6" s="2">
-        <v>58053</v>
+        <v>122632</v>
       </c>
       <c r="D6" s="1">
         <f t="shared" si="0"/>
-        <v>6.9040359671334817E-2</v>
+        <v>7.6146519668602003E-2</v>
       </c>
       <c r="E6" s="4">
-        <f>C6/$C$7</f>
-        <v>2.6014921620934904E-2</v>
+        <f>C6/$C$9</f>
+        <v>5.4978836877855541E-2</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="9" t="s">
+      <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="2">
+        <v>5455</v>
+      </c>
+      <c r="C7" s="2">
+        <v>65903</v>
+      </c>
+      <c r="D7" s="1">
+        <f t="shared" si="0"/>
+        <v>8.2773166623674191E-2</v>
+      </c>
+      <c r="E7" s="4">
+        <f>C7/$C$9</f>
+        <v>2.954587943408991E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="2">
+        <f>B6-B7</f>
+        <v>3883</v>
+      </c>
+      <c r="C8" s="2">
+        <f>C6-C7</f>
+        <v>56729</v>
+      </c>
+      <c r="D8" s="1">
+        <f t="shared" ref="D8" si="1">B8/C8</f>
+        <v>6.8448236351777755E-2</v>
+      </c>
+      <c r="E8" s="4">
+        <f>C8/$C$9</f>
+        <v>2.5432957443765631E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="10">
+      <c r="B9" s="10">
         <f>B6+B5+B2</f>
-        <v>177704</v>
-      </c>
-      <c r="C7" s="10">
+        <v>177689</v>
+      </c>
+      <c r="C9" s="10">
         <f>C6+C5+C2</f>
-        <v>2231527</v>
-      </c>
-      <c r="D7" s="11">
+        <v>2230531</v>
+      </c>
+      <c r="D9" s="11">
         <f t="shared" si="0"/>
-        <v>7.963336316343024E-2</v>
-      </c>
-      <c r="E7" s="9"/>
+        <v>7.9662197028420589E-2</v>
+      </c>
+      <c r="E9" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add ecoregion trends by owner
</commit_message>
<xml_diff>
--- a/tables/ownership_summary.xlsx
+++ b/tables/ownership_summary.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20406"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20407"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\ORISE\Projects\salvage\pfh\tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BF14C29-BE0F-43DA-90F0-9B3CDF0D9979}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C2CAF87-3217-44D6-A468-D0DB4CF217A7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="7980" xr2:uid="{7179679D-7B0A-430B-92F9-F823978B3D0B}"/>
   </bookViews>
@@ -75,7 +75,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -84,6 +84,14 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -99,7 +107,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -118,34 +126,50 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -473,174 +497,174 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="3">
+        <v>1632784</v>
+      </c>
+      <c r="C2" s="3">
         <v>79815</v>
       </c>
-      <c r="C2" s="2">
-        <v>1632784</v>
-      </c>
-      <c r="D2" s="1">
-        <f>B2/C2</f>
+      <c r="D2" s="4">
+        <f>C2/B2</f>
         <v>4.8882767102078416E-2</v>
       </c>
-      <c r="E2" s="4">
-        <f>C2/$C$9</f>
+      <c r="E2" s="5">
+        <f>B2/$B$9</f>
         <v>0.7320158294146103</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="9" t="s">
         <v>6</v>
       </c>
       <c r="B3" s="6">
+        <v>1457159</v>
+      </c>
+      <c r="C3" s="6">
         <v>71690</v>
       </c>
-      <c r="C3" s="6">
-        <v>1457159</v>
-      </c>
       <c r="D3" s="7">
-        <f t="shared" ref="D3:D9" si="0">B3/C3</f>
+        <f>C3/B3</f>
         <v>4.9198474565919026E-2</v>
       </c>
       <c r="E3" s="8">
-        <f>C3/$C$9</f>
+        <f>B3/$B$9</f>
         <v>0.65327897258545164</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="9" t="s">
         <v>7</v>
       </c>
       <c r="B4" s="6">
+        <v>174431</v>
+      </c>
+      <c r="C4" s="6">
         <v>8097</v>
       </c>
-      <c r="C4" s="6">
-        <v>174431</v>
-      </c>
       <c r="D4" s="7">
-        <f t="shared" si="0"/>
+        <f>C4/B4</f>
         <v>4.6419501120787014E-2</v>
       </c>
       <c r="E4" s="8">
-        <f>C4/$C$9</f>
+        <f>B4/$B$9</f>
         <v>7.8201558283655326E-2</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="3">
+        <v>475115</v>
+      </c>
+      <c r="C5" s="3">
         <v>88536</v>
       </c>
-      <c r="C5" s="2">
-        <v>475115</v>
-      </c>
-      <c r="D5" s="1">
-        <f>B5/C5</f>
+      <c r="D5" s="4">
+        <f>C5/B5</f>
         <v>0.18634646348778716</v>
       </c>
-      <c r="E5" s="4">
-        <f>C5/$C$9</f>
+      <c r="E5" s="5">
+        <f>B5/$B$9</f>
         <v>0.21300533370753422</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="A6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6" s="3">
+        <v>122632</v>
+      </c>
+      <c r="C6" s="3">
         <v>9338</v>
       </c>
-      <c r="C6" s="2">
-        <v>122632</v>
-      </c>
-      <c r="D6" s="1">
-        <f t="shared" si="0"/>
+      <c r="D6" s="4">
+        <f>C6/B6</f>
         <v>7.6146519668602003E-2</v>
       </c>
-      <c r="E6" s="4">
-        <f>C6/$C$9</f>
+      <c r="E6" s="5">
+        <f>B6/$B$9</f>
         <v>5.4978836877855541E-2</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="A7" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7" s="3">
+        <v>65903</v>
+      </c>
+      <c r="C7" s="3">
         <v>5455</v>
       </c>
-      <c r="C7" s="2">
-        <v>65903</v>
-      </c>
-      <c r="D7" s="1">
-        <f t="shared" si="0"/>
+      <c r="D7" s="4">
+        <f>C7/B7</f>
         <v>8.2773166623674191E-2</v>
       </c>
-      <c r="E7" s="4">
-        <f>C7/$C$9</f>
+      <c r="E7" s="5">
+        <f>B7/$B$9</f>
         <v>2.954587943408991E-2</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="A8" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="2">
+      <c r="B8" s="3">
         <f>B6-B7</f>
+        <v>56729</v>
+      </c>
+      <c r="C8" s="3">
+        <f>C6-C7</f>
         <v>3883</v>
       </c>
-      <c r="C8" s="2">
-        <f>C6-C7</f>
-        <v>56729</v>
-      </c>
-      <c r="D8" s="1">
-        <f t="shared" ref="D8" si="1">B8/C8</f>
+      <c r="D8" s="4">
+        <f>C8/B8</f>
         <v>6.8448236351777755E-2</v>
       </c>
-      <c r="E8" s="4">
-        <f>C8/$C$9</f>
+      <c r="E8" s="5">
+        <f>B8/$B$9</f>
         <v>2.5432957443765631E-2</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="9" t="s">
+      <c r="A9" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="10">
+      <c r="B9" s="11">
         <f>B6+B5+B2</f>
+        <v>2230531</v>
+      </c>
+      <c r="C9" s="11">
+        <f>C6+C5+C2</f>
         <v>177689</v>
       </c>
-      <c r="C9" s="10">
-        <f>C6+C5+C2</f>
-        <v>2230531</v>
-      </c>
-      <c r="D9" s="11">
-        <f t="shared" si="0"/>
+      <c r="D9" s="12">
+        <f>C9/B9</f>
         <v>7.9662197028420589E-2</v>
       </c>
-      <c r="E9" s="9"/>
+      <c r="E9" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>